<commit_message>
Atualiza Excel professores com aba Cenários conselho
Co-authored-by: cbrener89052 <cbrener89052@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/professores_comuns_reuniao_C_2026.xlsx
+++ b/professores_comuns_reuniao_C_2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="7C+8C vs 11C+12C" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="6C-7C vs 9C-10C" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="5C-8C vs 11C-12C" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cenários conselho" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +37,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,16 +47,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D0E0E3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,12 +90,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,13 +465,13 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Professor</t>
@@ -545,7 +530,7 @@
       <c r="C2" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -588,7 +573,7 @@
       <c r="C3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -631,7 +616,7 @@
       <c r="C4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -674,7 +659,7 @@
       <c r="C5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -717,7 +702,7 @@
       <c r="C6" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -760,7 +745,7 @@
       <c r="C7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -803,7 +788,7 @@
       <c r="C8" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -846,7 +831,7 @@
       <c r="C9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -889,7 +874,7 @@
       <c r="C10" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -932,7 +917,7 @@
       <c r="C11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -975,7 +960,7 @@
       <c r="C12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1018,7 +1003,7 @@
       <c r="C13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1061,7 +1046,7 @@
       <c r="C14" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1104,7 +1089,7 @@
       <c r="C15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1147,7 +1132,7 @@
       <c r="C16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1190,7 +1175,7 @@
       <c r="C17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1233,7 +1218,7 @@
       <c r="C18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1276,7 +1261,7 @@
       <c r="C19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1319,7 +1304,7 @@
       <c r="C20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1362,7 +1347,7 @@
       <c r="C21" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1405,7 +1390,7 @@
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1448,7 +1433,7 @@
       <c r="C23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1491,7 +1476,7 @@
       <c r="C24" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1534,7 +1519,7 @@
       <c r="C25" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1577,7 +1562,7 @@
       <c r="C26" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1620,7 +1605,7 @@
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1663,7 +1648,7 @@
       <c r="C28" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1706,7 +1691,7 @@
       <c r="C29" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1749,7 +1734,7 @@
       <c r="C30" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1792,7 +1777,7 @@
       <c r="C31" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1835,7 +1820,7 @@
       <c r="C32" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1878,7 +1863,7 @@
       <c r="C33" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1921,7 +1906,7 @@
       <c r="C34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1964,7 +1949,7 @@
       <c r="C35" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2007,7 +1992,7 @@
       <c r="C36" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2050,7 +2035,7 @@
       <c r="C37" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2093,7 +2078,7 @@
       <c r="C38" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2136,7 +2121,7 @@
       <c r="C39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2179,7 +2164,7 @@
       <c r="C40" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2222,7 +2207,7 @@
       <c r="C41" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2265,7 +2250,7 @@
       <c r="C42" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2308,7 +2293,7 @@
       <c r="C43" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2351,7 +2336,7 @@
       <c r="C44" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2394,7 +2379,7 @@
       <c r="C45" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2437,7 +2422,7 @@
       <c r="C46" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2480,7 +2465,7 @@
       <c r="C47" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2523,7 +2508,7 @@
       <c r="C48" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2566,7 +2551,7 @@
       <c r="C49" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2609,7 +2594,7 @@
       <c r="C50" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2652,7 +2637,7 @@
       <c r="C51" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2695,7 +2680,7 @@
       <c r="C52" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2738,7 +2723,7 @@
       <c r="C53" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2781,7 +2766,7 @@
       <c r="C54" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2824,7 +2809,7 @@
       <c r="C55" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2867,7 +2852,7 @@
       <c r="C56" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2910,7 +2895,7 @@
       <c r="C57" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2953,7 +2938,7 @@
       <c r="C58" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2996,7 +2981,7 @@
       <c r="C59" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3039,7 +3024,7 @@
       <c r="C60" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3082,7 +3067,7 @@
       <c r="C61" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3125,7 +3110,7 @@
       <c r="C62" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3168,7 +3153,7 @@
       <c r="C63" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3211,7 +3196,7 @@
       <c r="C64" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Empate</t>
         </is>
@@ -3254,7 +3239,7 @@
       <c r="C65" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3297,7 +3282,7 @@
       <c r="C66" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3340,7 +3325,7 @@
       <c r="C67" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3392,17 +3377,17 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Segmento</t>
@@ -3490,7 +3475,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3506,7 +3491,7 @@
       <c r="F2" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3547,7 +3532,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3563,7 +3548,7 @@
       <c r="F3" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3604,7 +3589,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3620,7 +3605,7 @@
       <c r="F4" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3661,7 +3646,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3677,7 +3662,7 @@
       <c r="F5" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3718,7 +3703,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3734,7 +3719,7 @@
       <c r="F6" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3775,7 +3760,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -3791,7 +3776,7 @@
       <c r="F7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -3832,7 +3817,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3848,7 +3833,7 @@
       <c r="F8" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3889,7 +3874,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3905,7 +3890,7 @@
       <c r="F9" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3946,7 +3931,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -3962,7 +3947,7 @@
       <c r="F10" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4003,7 +3988,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4019,7 +4004,7 @@
       <c r="F11" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4060,7 +4045,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4076,7 +4061,7 @@
       <c r="F12" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4117,7 +4102,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4133,7 +4118,7 @@
       <c r="F13" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4174,7 +4159,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4190,7 +4175,7 @@
       <c r="F14" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4231,7 +4216,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4247,7 +4232,7 @@
       <c r="F15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4288,7 +4273,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -4304,7 +4289,7 @@
       <c r="F16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -4345,7 +4330,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4361,7 +4346,7 @@
       <c r="F17" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4402,7 +4387,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4418,7 +4403,7 @@
       <c r="F18" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4459,7 +4444,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -4475,7 +4460,7 @@
       <c r="F19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -4516,7 +4501,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4532,7 +4517,7 @@
       <c r="F20" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4573,7 +4558,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4589,7 +4574,7 @@
       <c r="F21" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4630,7 +4615,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -4646,7 +4631,7 @@
       <c r="F22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -4687,7 +4672,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4703,7 +4688,7 @@
       <c r="F23" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4744,7 +4729,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4760,7 +4745,7 @@
       <c r="F24" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4801,7 +4786,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -4817,7 +4802,7 @@
       <c r="F25" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -4858,7 +4843,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -4874,7 +4859,7 @@
       <c r="F26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -4915,7 +4900,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -4931,7 +4916,7 @@
       <c r="F27" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -4972,7 +4957,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -4988,7 +4973,7 @@
       <c r="F28" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5029,7 +5014,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5045,7 +5030,7 @@
       <c r="F29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5086,7 +5071,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5102,7 +5087,7 @@
       <c r="F30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5143,7 +5128,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5159,7 +5144,7 @@
       <c r="F31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5200,7 +5185,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -5216,7 +5201,7 @@
       <c r="F32" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5257,7 +5242,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -5273,7 +5258,7 @@
       <c r="F33" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5314,7 +5299,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5330,7 +5315,7 @@
       <c r="F34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5371,7 +5356,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -5387,7 +5372,7 @@
       <c r="F35" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5428,7 +5413,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -5444,7 +5429,7 @@
       <c r="F36" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5485,7 +5470,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -5501,7 +5486,7 @@
       <c r="F37" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5542,7 +5527,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5558,7 +5543,7 @@
       <c r="F38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5599,7 +5584,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -5615,7 +5600,7 @@
       <c r="F39" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5656,7 +5641,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5672,7 +5657,7 @@
       <c r="F40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5713,7 +5698,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -5729,7 +5714,7 @@
       <c r="F41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -5770,7 +5755,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -5786,7 +5771,7 @@
       <c r="F42" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5827,7 +5812,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -5843,7 +5828,7 @@
       <c r="F43" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5884,7 +5869,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -5900,7 +5885,7 @@
       <c r="F44" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5941,7 +5926,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -5957,7 +5942,7 @@
       <c r="F45" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5998,7 +5983,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6014,7 +5999,7 @@
       <c r="F46" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6055,7 +6040,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6071,7 +6056,7 @@
       <c r="F47" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6112,7 +6097,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -6128,7 +6113,7 @@
       <c r="F48" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6169,7 +6154,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -6185,7 +6170,7 @@
       <c r="F49" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="G49" s="4" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6226,7 +6211,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -6242,7 +6227,7 @@
       <c r="F50" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6283,7 +6268,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6299,7 +6284,7 @@
       <c r="F51" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6340,7 +6325,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -6356,7 +6341,7 @@
       <c r="F52" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6397,7 +6382,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -6413,7 +6398,7 @@
       <c r="F53" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6454,7 +6439,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -6470,7 +6455,7 @@
       <c r="F54" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6511,7 +6496,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -6527,7 +6512,7 @@
       <c r="F55" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6568,7 +6553,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -6584,7 +6569,7 @@
       <c r="F56" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6625,7 +6610,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6641,7 +6626,7 @@
       <c r="F57" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6682,7 +6667,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6698,7 +6683,7 @@
       <c r="F58" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6739,7 +6724,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6755,7 +6740,7 @@
       <c r="F59" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6796,7 +6781,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -6812,7 +6797,7 @@
       <c r="F60" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G60" s="4" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6853,7 +6838,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6869,7 +6854,7 @@
       <c r="F61" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6910,7 +6895,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -6926,7 +6911,7 @@
       <c r="F62" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G62" s="4" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -6967,7 +6952,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -6983,7 +6968,7 @@
       <c r="F63" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7024,7 +7009,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7040,7 +7025,7 @@
       <c r="F64" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7081,7 +7066,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -7097,7 +7082,7 @@
       <c r="F65" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G65" s="4" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -7138,7 +7123,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -7195,7 +7180,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7211,7 +7196,7 @@
       <c r="F67" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G67" s="3" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7252,7 +7237,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7268,7 +7253,7 @@
       <c r="F68" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7309,7 +7294,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7325,7 +7310,7 @@
       <c r="F69" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G69" s="3" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7366,7 +7351,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7382,7 +7367,7 @@
       <c r="F70" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7423,7 +7408,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -7439,7 +7424,7 @@
       <c r="F71" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G71" s="4" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -7480,7 +7465,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -7496,7 +7481,7 @@
       <c r="F72" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G72" s="4" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -7537,7 +7522,7 @@
           <t>5-8</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -7553,7 +7538,7 @@
       <c r="F73" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G73" s="4" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -7594,7 +7579,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7606,7 +7591,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="3" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7651,7 +7636,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -7663,7 +7648,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="4" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -7708,7 +7693,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -7720,7 +7705,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="3" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7765,7 +7750,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -7777,7 +7762,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="3" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7822,7 +7807,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7834,7 +7819,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="3" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7879,7 +7864,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -7891,7 +7876,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="3" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -7936,7 +7921,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -7948,7 +7933,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="G80" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -7993,7 +7978,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8005,7 +7990,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="4" t="inlineStr">
+      <c r="G81" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8050,7 +8035,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8062,7 +8047,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8107,7 +8092,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8119,7 +8104,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" s="4" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8164,7 +8149,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8176,7 +8161,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="3" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8221,7 +8206,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8233,7 +8218,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="4" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8278,7 +8263,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -8290,7 +8275,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="3" t="inlineStr">
+      <c r="G86" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8335,7 +8320,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C87" s="3" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8347,7 +8332,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" s="3" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8392,7 +8377,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -8404,7 +8389,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="3" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8449,7 +8434,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C89" s="4" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8461,7 +8446,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="4" t="inlineStr">
+      <c r="G89" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8506,7 +8491,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8518,7 +8503,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="4" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8563,7 +8548,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C91" s="3" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8575,7 +8560,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" s="3" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8620,7 +8605,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C92" s="3" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8632,7 +8617,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="3" t="inlineStr">
+      <c r="G92" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8677,7 +8662,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8689,7 +8674,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr"/>
       <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="3" t="inlineStr">
+      <c r="G93" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8734,7 +8719,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C94" s="3" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8746,7 +8731,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" s="3" t="inlineStr">
+      <c r="G94" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8791,7 +8776,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C95" s="3" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8803,7 +8788,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="3" t="inlineStr">
+      <c r="G95" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8848,7 +8833,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C96" s="3" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8860,7 +8845,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="3" t="inlineStr">
+      <c r="G96" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -8905,7 +8890,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -8917,7 +8902,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="4" t="inlineStr">
+      <c r="G97" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -8962,7 +8947,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C98" s="3" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -8974,7 +8959,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="3" t="inlineStr">
+      <c r="G98" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9019,7 +9004,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9031,7 +9016,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="3" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9076,7 +9061,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -9088,7 +9073,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr"/>
       <c r="F100" s="2" t="inlineStr"/>
-      <c r="G100" s="4" t="inlineStr">
+      <c r="G100" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9133,7 +9118,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9145,7 +9130,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr"/>
-      <c r="G101" s="3" t="inlineStr">
+      <c r="G101" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9190,7 +9175,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C102" s="3" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -9202,7 +9187,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr"/>
       <c r="F102" s="2" t="inlineStr"/>
-      <c r="G102" s="3" t="inlineStr">
+      <c r="G102" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9247,7 +9232,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C103" s="4" t="inlineStr">
+      <c r="C103" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -9259,7 +9244,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr"/>
       <c r="F103" s="2" t="inlineStr"/>
-      <c r="G103" s="4" t="inlineStr">
+      <c r="G103" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9304,7 +9289,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C104" s="4" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -9316,7 +9301,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" s="4" t="inlineStr">
+      <c r="G104" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9361,7 +9346,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C105" s="3" t="inlineStr">
+      <c r="C105" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -9373,7 +9358,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="inlineStr"/>
-      <c r="G105" s="3" t="inlineStr">
+      <c r="G105" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9418,7 +9403,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C106" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9430,7 +9415,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr"/>
       <c r="F106" s="2" t="inlineStr"/>
-      <c r="G106" s="4" t="inlineStr">
+      <c r="G106" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9475,7 +9460,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C107" s="5" t="inlineStr">
+      <c r="C107" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9487,7 +9472,7 @@
       </c>
       <c r="E107" s="2" t="inlineStr"/>
       <c r="F107" s="2" t="inlineStr"/>
-      <c r="G107" s="3" t="inlineStr">
+      <c r="G107" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9532,7 +9517,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C108" s="4" t="inlineStr">
+      <c r="C108" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -9544,7 +9529,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr"/>
-      <c r="G108" s="4" t="inlineStr">
+      <c r="G108" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9589,7 +9574,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C109" s="5" t="inlineStr">
+      <c r="C109" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9601,7 +9586,7 @@
       </c>
       <c r="E109" s="2" t="inlineStr"/>
       <c r="F109" s="2" t="inlineStr"/>
-      <c r="G109" s="4" t="inlineStr">
+      <c r="G109" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9646,7 +9631,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C110" s="5" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9703,7 +9688,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C111" s="4" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -9715,7 +9700,7 @@
       </c>
       <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr"/>
-      <c r="G111" s="4" t="inlineStr">
+      <c r="G111" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9760,7 +9745,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C112" s="5" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9772,7 +9757,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" s="3" t="inlineStr">
+      <c r="G112" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9817,7 +9802,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C113" s="3" t="inlineStr">
+      <c r="C113" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -9829,7 +9814,7 @@
       </c>
       <c r="E113" s="2" t="inlineStr"/>
       <c r="F113" s="2" t="inlineStr"/>
-      <c r="G113" s="3" t="inlineStr">
+      <c r="G113" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -9874,7 +9859,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C114" s="4" t="inlineStr">
+      <c r="C114" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -9886,7 +9871,7 @@
       </c>
       <c r="E114" s="2" t="inlineStr"/>
       <c r="F114" s="2" t="inlineStr"/>
-      <c r="G114" s="4" t="inlineStr">
+      <c r="G114" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -9931,7 +9916,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C115" s="5" t="inlineStr">
+      <c r="C115" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -9988,7 +9973,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C116" s="3" t="inlineStr">
+      <c r="C116" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10000,7 +9985,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr"/>
       <c r="F116" s="2" t="inlineStr"/>
-      <c r="G116" s="3" t="inlineStr">
+      <c r="G116" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10045,7 +10030,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C117" s="5" t="inlineStr">
+      <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10057,7 +10042,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr"/>
       <c r="F117" s="2" t="inlineStr"/>
-      <c r="G117" s="4" t="inlineStr">
+      <c r="G117" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -10102,7 +10087,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C118" s="5" t="inlineStr">
+      <c r="C118" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10114,7 +10099,7 @@
       </c>
       <c r="E118" s="2" t="inlineStr"/>
       <c r="F118" s="2" t="inlineStr"/>
-      <c r="G118" s="4" t="inlineStr">
+      <c r="G118" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -10159,7 +10144,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C119" s="5" t="inlineStr">
+      <c r="C119" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10171,7 +10156,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr"/>
       <c r="F119" s="2" t="inlineStr"/>
-      <c r="G119" s="3" t="inlineStr">
+      <c r="G119" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10216,7 +10201,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C120" s="5" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10228,7 +10213,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr"/>
       <c r="F120" s="2" t="inlineStr"/>
-      <c r="G120" s="3" t="inlineStr">
+      <c r="G120" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10273,7 +10258,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C121" s="5" t="inlineStr">
+      <c r="C121" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10330,7 +10315,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C122" s="3" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10342,7 +10327,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr"/>
       <c r="F122" s="2" t="inlineStr"/>
-      <c r="G122" s="3" t="inlineStr">
+      <c r="G122" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10387,7 +10372,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C123" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10399,7 +10384,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr"/>
       <c r="F123" s="2" t="inlineStr"/>
-      <c r="G123" s="3" t="inlineStr">
+      <c r="G123" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10444,7 +10429,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C124" s="3" t="inlineStr">
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10456,7 +10441,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr"/>
       <c r="F124" s="2" t="inlineStr"/>
-      <c r="G124" s="3" t="inlineStr">
+      <c r="G124" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10501,7 +10486,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C125" s="5" t="inlineStr">
+      <c r="C125" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10513,7 +10498,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr"/>
-      <c r="G125" s="3" t="inlineStr">
+      <c r="G125" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10558,7 +10543,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C126" s="4" t="inlineStr">
+      <c r="C126" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -10570,7 +10555,7 @@
       </c>
       <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr"/>
-      <c r="G126" s="4" t="inlineStr">
+      <c r="G126" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -10615,7 +10600,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C127" s="4" t="inlineStr">
+      <c r="C127" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -10627,7 +10612,7 @@
       </c>
       <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr"/>
-      <c r="G127" s="4" t="inlineStr">
+      <c r="G127" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -10672,7 +10657,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C128" s="3" t="inlineStr">
+      <c r="C128" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10684,7 +10669,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr"/>
       <c r="F128" s="2" t="inlineStr"/>
-      <c r="G128" s="3" t="inlineStr">
+      <c r="G128" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10729,7 +10714,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C129" s="3" t="inlineStr">
+      <c r="C129" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10741,7 +10726,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr"/>
       <c r="F129" s="2" t="inlineStr"/>
-      <c r="G129" s="3" t="inlineStr">
+      <c r="G129" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10786,7 +10771,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C130" s="3" t="inlineStr">
+      <c r="C130" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10798,7 +10783,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr"/>
-      <c r="G130" s="3" t="inlineStr">
+      <c r="G130" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10843,7 +10828,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C131" s="3" t="inlineStr">
+      <c r="C131" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -10855,7 +10840,7 @@
       </c>
       <c r="E131" s="2" t="inlineStr"/>
       <c r="F131" s="2" t="inlineStr"/>
-      <c r="G131" s="3" t="inlineStr">
+      <c r="G131" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -10900,7 +10885,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C132" s="5" t="inlineStr">
+      <c r="C132" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -10912,7 +10897,7 @@
       </c>
       <c r="E132" s="2" t="inlineStr"/>
       <c r="F132" s="2" t="inlineStr"/>
-      <c r="G132" s="4" t="inlineStr">
+      <c r="G132" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -10957,7 +10942,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C133" s="4" t="inlineStr">
+      <c r="C133" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -10969,7 +10954,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr"/>
       <c r="F133" s="2" t="inlineStr"/>
-      <c r="G133" s="4" t="inlineStr">
+      <c r="G133" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -11014,7 +10999,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C134" s="5" t="inlineStr">
+      <c r="C134" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -11071,7 +11056,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C135" s="3" t="inlineStr">
+      <c r="C135" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -11083,7 +11068,7 @@
       </c>
       <c r="E135" s="2" t="inlineStr"/>
       <c r="F135" s="2" t="inlineStr"/>
-      <c r="G135" s="3" t="inlineStr">
+      <c r="G135" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -11128,7 +11113,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C136" s="3" t="inlineStr">
+      <c r="C136" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -11140,7 +11125,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr"/>
       <c r="F136" s="2" t="inlineStr"/>
-      <c r="G136" s="3" t="inlineStr">
+      <c r="G136" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -11185,7 +11170,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C137" s="3" t="inlineStr">
+      <c r="C137" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -11197,7 +11182,7 @@
       </c>
       <c r="E137" s="2" t="inlineStr"/>
       <c r="F137" s="2" t="inlineStr"/>
-      <c r="G137" s="3" t="inlineStr">
+      <c r="G137" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -11242,7 +11227,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C138" s="4" t="inlineStr">
+      <c r="C138" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -11254,7 +11239,7 @@
       </c>
       <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr"/>
-      <c r="G138" s="4" t="inlineStr">
+      <c r="G138" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -11299,7 +11284,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
+      <c r="C139" s="2" t="inlineStr">
         <is>
           <t>Só R</t>
         </is>
@@ -11311,7 +11296,7 @@
       </c>
       <c r="E139" s="2" t="inlineStr"/>
       <c r="F139" s="2" t="inlineStr"/>
-      <c r="G139" s="4" t="inlineStr">
+      <c r="G139" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
@@ -11356,7 +11341,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C140" s="3" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -11368,7 +11353,7 @@
       </c>
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr"/>
-      <c r="G140" s="3" t="inlineStr">
+      <c r="G140" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -11413,7 +11398,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C141" s="3" t="inlineStr">
+      <c r="C141" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -11425,7 +11410,7 @@
       </c>
       <c r="E141" s="2" t="inlineStr"/>
       <c r="F141" s="2" t="inlineStr"/>
-      <c r="G141" s="3" t="inlineStr">
+      <c r="G141" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -11470,7 +11455,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C142" s="5" t="inlineStr">
+      <c r="C142" s="2" t="inlineStr">
         <is>
           <t>Comum</t>
         </is>
@@ -11527,7 +11512,7 @@
           <t>9-12</t>
         </is>
       </c>
-      <c r="C143" s="3" t="inlineStr">
+      <c r="C143" s="2" t="inlineStr">
         <is>
           <t>Só C</t>
         </is>
@@ -11539,7 +11524,7 @@
       </c>
       <c r="E143" s="2" t="inlineStr"/>
       <c r="F143" s="2" t="inlineStr"/>
-      <c r="G143" s="3" t="inlineStr">
+      <c r="G143" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -11589,20 +11574,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -11686,7 +11671,7 @@
       <c r="D2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -11749,7 +11734,7 @@
       <c r="D3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -11812,7 +11797,7 @@
       <c r="D4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -11875,7 +11860,7 @@
       <c r="D5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -11938,7 +11923,7 @@
       <c r="D6" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12001,7 +11986,7 @@
       <c r="D7" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12064,7 +12049,7 @@
       <c r="D8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -12127,7 +12112,7 @@
       <c r="D9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12190,7 +12175,7 @@
       <c r="D10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12253,7 +12238,7 @@
       <c r="D11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12316,7 +12301,7 @@
       <c r="D12" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12379,7 +12364,7 @@
       <c r="D13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12442,7 +12427,7 @@
       <c r="D14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12505,7 +12490,7 @@
       <c r="D15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12568,7 +12553,7 @@
       <c r="D16" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12631,7 +12616,7 @@
       <c r="D17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12694,7 +12679,7 @@
       <c r="D18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12757,7 +12742,7 @@
       <c r="D19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12820,7 +12805,7 @@
       <c r="D20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -12883,7 +12868,7 @@
       <c r="D21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -12946,7 +12931,7 @@
       <c r="D22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13009,7 +12994,7 @@
       <c r="D23" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13072,7 +13057,7 @@
       <c r="D24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13135,7 +13120,7 @@
       <c r="D25" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -13198,7 +13183,7 @@
       <c r="D26" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13261,7 +13246,7 @@
       <c r="D27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -13324,7 +13309,7 @@
       <c r="D28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13387,7 +13372,7 @@
       <c r="D29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13450,7 +13435,7 @@
       <c r="D30" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13513,7 +13498,7 @@
       <c r="D31" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13576,7 +13561,7 @@
       <c r="D32" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -13639,7 +13624,7 @@
       <c r="D33" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13702,7 +13687,7 @@
       <c r="D34" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13765,7 +13750,7 @@
       <c r="D35" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -13828,7 +13813,7 @@
       <c r="D36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -13891,7 +13876,7 @@
       <c r="D37" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -13954,7 +13939,7 @@
       <c r="D38" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14017,7 +14002,7 @@
       <c r="D39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14079,20 +14064,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="39" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -14176,7 +14161,7 @@
       <c r="D2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14239,7 +14224,7 @@
       <c r="D3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14302,7 +14287,7 @@
       <c r="D4" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14365,7 +14350,7 @@
       <c r="D5" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14428,7 +14413,7 @@
       <c r="D6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14491,7 +14476,7 @@
       <c r="D7" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14554,7 +14539,7 @@
       <c r="D8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14617,7 +14602,7 @@
       <c r="D9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14680,7 +14665,7 @@
       <c r="D10" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14743,7 +14728,7 @@
       <c r="D11" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -14806,7 +14791,7 @@
       <c r="D12" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14869,7 +14854,7 @@
       <c r="D13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14932,7 +14917,7 @@
       <c r="D14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -14995,7 +14980,7 @@
       <c r="D15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15058,7 +15043,7 @@
       <c r="D16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15121,7 +15106,7 @@
       <c r="D17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15184,7 +15169,7 @@
       <c r="D18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -15247,7 +15232,7 @@
       <c r="D19" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15310,7 +15295,7 @@
       <c r="D20" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15373,7 +15358,7 @@
       <c r="D21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15436,7 +15421,7 @@
       <c r="D22" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -15499,7 +15484,7 @@
       <c r="D23" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15562,7 +15547,7 @@
       <c r="D24" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15625,7 +15610,7 @@
       <c r="D25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -15688,7 +15673,7 @@
       <c r="D26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15751,7 +15736,7 @@
       <c r="D27" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -15814,7 +15799,7 @@
       <c r="D28" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15877,7 +15862,7 @@
       <c r="D29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -15940,7 +15925,7 @@
       <c r="D30" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16002,20 +15987,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -16099,7 +16084,7 @@
       <c r="D2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -16162,7 +16147,7 @@
       <c r="D3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -16225,7 +16210,7 @@
       <c r="D4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -16288,7 +16273,7 @@
       <c r="D5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16351,7 +16336,7 @@
       <c r="D6" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16414,7 +16399,7 @@
       <c r="D7" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16477,7 +16462,7 @@
       <c r="D8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16540,7 +16525,7 @@
       <c r="D9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16603,7 +16588,7 @@
       <c r="D10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16666,7 +16651,7 @@
       <c r="D11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16729,7 +16714,7 @@
       <c r="D12" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16792,7 +16777,7 @@
       <c r="D13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16855,7 +16840,7 @@
       <c r="D14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -16918,7 +16903,7 @@
       <c r="D15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -16981,7 +16966,7 @@
       <c r="D16" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17044,7 +17029,7 @@
       <c r="D17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17107,7 +17092,7 @@
       <c r="D18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17170,7 +17155,7 @@
       <c r="D19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17233,7 +17218,7 @@
       <c r="D20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17296,7 +17281,7 @@
       <c r="D21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17359,7 +17344,7 @@
       <c r="D22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17422,7 +17407,7 @@
       <c r="D23" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17485,7 +17470,7 @@
       <c r="D24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17548,7 +17533,7 @@
       <c r="D25" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -17611,7 +17596,7 @@
       <c r="D26" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17674,7 +17659,7 @@
       <c r="D27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -17737,7 +17722,7 @@
       <c r="D28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17800,7 +17785,7 @@
       <c r="D29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17863,7 +17848,7 @@
       <c r="D30" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -17926,7 +17911,7 @@
       <c r="D31" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -17989,7 +17974,7 @@
       <c r="D32" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18052,7 +18037,7 @@
       <c r="D33" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18115,7 +18100,7 @@
       <c r="D34" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18178,7 +18163,7 @@
       <c r="D35" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18241,7 +18226,7 @@
       <c r="D36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18304,7 +18289,7 @@
       <c r="D37" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18367,7 +18352,7 @@
       <c r="D38" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18430,7 +18415,7 @@
       <c r="D39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18492,20 +18477,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -18589,7 +18574,7 @@
       <c r="D2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18652,7 +18637,7 @@
       <c r="D3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18715,7 +18700,7 @@
       <c r="D4" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18778,7 +18763,7 @@
       <c r="D5" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18841,7 +18826,7 @@
       <c r="D6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -18904,7 +18889,7 @@
       <c r="D7" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -18967,7 +18952,7 @@
       <c r="D8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19030,7 +19015,7 @@
       <c r="D9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19093,7 +19078,7 @@
       <c r="D10" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19156,7 +19141,7 @@
       <c r="D11" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19219,7 +19204,7 @@
       <c r="D12" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19282,7 +19267,7 @@
       <c r="D13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19345,7 +19330,7 @@
       <c r="D14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19408,7 +19393,7 @@
       <c r="D15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19471,7 +19456,7 @@
       <c r="D16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19534,7 +19519,7 @@
       <c r="D17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -19597,7 +19582,7 @@
       <c r="D18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19660,7 +19645,7 @@
       <c r="D19" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19723,7 +19708,7 @@
       <c r="D20" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19786,7 +19771,7 @@
       <c r="D21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19849,7 +19834,7 @@
       <c r="D22" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -19912,7 +19897,7 @@
       <c r="D23" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -19975,7 +19960,7 @@
       <c r="D24" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -20038,7 +20023,7 @@
       <c r="D25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -20101,7 +20086,7 @@
       <c r="D26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -20164,7 +20149,7 @@
       <c r="D27" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -20227,7 +20212,7 @@
       <c r="D28" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -20290,7 +20275,7 @@
       <c r="D29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -20353,7 +20338,7 @@
       <c r="D30" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -20397,6 +20382,290 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cenário</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Bloco EFII</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Bloco EM</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Prof. no cenário</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Só EFII (livre)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Só EM (livre)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Comuns (conflito)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Comuns → EFII</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Comuns → EM</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Empates TL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Disponíveis conselho EFII</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Disponíveis conselho EM</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Saldo EFII − EM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>5-6 vs 9-10</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>5C+6C</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>9C+10C</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>6-7 vs 9-10</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>6C+7C</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>9C+10C</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>7-8 vs 9-10</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>7C+8C</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>9C+10C</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>6-7 vs 11-12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>6C+7C</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>11C+12C</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Inclui cenário 8-9 vs 11-12 na aba Cenários conselho
Adiciona linha 8C+9C vs 11C+12C com contagem de professores
disponíveis por bloco (28 conselho bloco 1, 24 conselho bloco 2).

Co-authored-by: cbrener89052 <cbrener89052@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/professores_comuns_reuniao_C_2026.xlsx
+++ b/professores_comuns_reuniao_C_2026.xlsx
@@ -51,7 +51,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -465,13 +465,13 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Professor</t>
@@ -3377,17 +3377,17 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Segmento</t>
@@ -11574,20 +11574,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -14064,20 +14064,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -15987,20 +15987,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -18477,20 +18477,20 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -20395,25 +20395,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cenário</t>
@@ -20421,12 +20421,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Bloco EFII</t>
+          <t>Bloco 1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Bloco EM</t>
+          <t>Bloco 2</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -20436,12 +20436,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Só EFII (livre)</t>
+          <t>Só bloco 1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Só EM (livre)</t>
+          <t>Só bloco 2</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -20451,12 +20451,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Comuns → EFII</t>
+          <t>Comuns → bloco 1</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Comuns → EM</t>
+          <t>Comuns → bloco 2</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -20466,17 +20466,17 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Disponíveis conselho EFII</t>
+          <t>Conselho bloco 1</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Disponíveis conselho EM</t>
+          <t>Conselho bloco 2</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Saldo EFII − EM</t>
+          <t>Saldo bloco1 − bloco2</t>
         </is>
       </c>
     </row>
@@ -20622,50 +20622,238 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>6-7 vs 11-12</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>6C+7C</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>11C+12C</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="3" t="n">
+      <c r="J5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="L5" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="M5" s="2" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>8-9 vs 11-12</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>8C+9C</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>11C+12C</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5-6 vs 11-12</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>5C+6C</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>11C+12C</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7-8 vs 11-12</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>7C+8C</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>11C+12C</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>5-8 vs 9-10</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>5C+8C</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>9C+10C</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>